<commit_message>
in case of shtd
</commit_message>
<xml_diff>
--- a/simulations/scene/inputs/Scenarios_25-11-01.xlsx
+++ b/simulations/scene/inputs/Scenarios_25-11-01.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TIGERA~1\AppData\Local\Temp\scp55262\work_home\tigerault\Wheat-BRIDGES_framework\Wheat-BRIDGES\simulations\scene\inputs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TIGERA~1\AppData\Local\Temp\scp29402\work_home\tigerault\Wheat-BRIDGES_framework\Wheat-BRIDGES\simulations\scene\inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DA96082-2C7E-4F83-9A7B-24093819C3B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54F8FA66-2408-4186-8F14-B8800CF1F467}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2968,7 +2968,7 @@
         <v>564</v>
       </c>
       <c r="K3" s="43" t="s">
-        <v>564</v>
+        <v>485</v>
       </c>
     </row>
     <row r="4" spans="1:47" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -9664,10 +9664,10 @@
         <v>0.25</v>
       </c>
       <c r="J209" s="43">
-        <v>0.25</v>
+        <v>0.31</v>
       </c>
       <c r="K209" s="43">
-        <v>0.25</v>
+        <v>0.31</v>
       </c>
       <c r="M209" s="50"/>
       <c r="N209" s="50"/>
@@ -10982,10 +10982,10 @@
         <v>0.1</v>
       </c>
       <c r="J239" s="43">
-        <v>0.1</v>
+        <v>0.01</v>
       </c>
       <c r="K239" s="43">
-        <v>0.1</v>
+        <v>0.01</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
final working version with adjustment of the vmax_AA_xylem, optimum x10 for RSA and leaf length
</commit_message>
<xml_diff>
--- a/simulations/scene/inputs/Scenarios_25-11-01.xlsx
+++ b/simulations/scene/inputs/Scenarios_25-11-01.xlsx
@@ -9608,8 +9608,8 @@
         <v>2.5E-011</v>
       </c>
       <c r="J216" s="10" t="n">
-        <f aca="false">0.0000000000025*10</f>
-        <v>2.5E-011</v>
+        <f aca="false">0.0000000000025</f>
+        <v>2.5E-012</v>
       </c>
       <c r="K216" s="10" t="n">
         <f aca="false">0.0000000000025*10</f>
@@ -9944,8 +9944,8 @@
         <v>1.2E-007</v>
       </c>
       <c r="J224" s="10" t="n">
-        <f aca="false">0.00001 / 10 / 5 / 10 * 6 * 100</f>
-        <v>1.2E-005</v>
+        <f aca="false">0.00001 / 10 / 5 / 10 * 6 * 5</f>
+        <v>6E-007</v>
       </c>
       <c r="K224" s="10" t="n">
         <f aca="false">0.00001 / 10 / 5 / 10 * 6</f>
@@ -10028,8 +10028,8 @@
         <v>1.2E-005</v>
       </c>
       <c r="J226" s="10" t="n">
-        <f aca="false">0.00001 /5 /2/4 * 4 * 0.6 * 10*2</f>
-        <v>1.2E-005</v>
+        <f aca="false">0.00001 /5 /2/4 * 4 * 0.6 * 10*2 * 50</f>
+        <v>0.0006</v>
       </c>
       <c r="K226" s="10" t="n">
         <f aca="false">0.00001 /5 /2/4 * 4 * 0.6 * 10*2</f>

</xml_diff>